<commit_message>
Updated moments of inertia of major components
</commit_message>
<xml_diff>
--- a/HER04/mass_input_cfg_1.xlsx
+++ b/HER04/mass_input_cfg_1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ash\Documents\University Files\Year 3\GDP\gdp_repo\HER04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5177771-F790-4CCC-80CD-E75FECC9F67D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{C7DA80BD-D061-42D7-B3A5-ED80209841BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>Component</t>
   </si>
@@ -74,9 +75,6 @@
     <t>Fuel Tanks</t>
   </si>
   <si>
-    <t>Elec, Hyd</t>
-  </si>
-  <si>
     <t>Battery</t>
   </si>
   <si>
@@ -147,6 +145,15 @@
   </si>
   <si>
     <t>Passenger Jumpseat</t>
+  </si>
+  <si>
+    <t>Hydraulics</t>
+  </si>
+  <si>
+    <t>Generators</t>
+  </si>
+  <si>
+    <t>Electrical Cabling</t>
   </si>
 </sst>
 </file>
@@ -464,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51.26953125" bestFit="1" customWidth="1"/>
@@ -507,10 +514,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B2">
-        <v>195.61080000000001</v>
+        <v>302</v>
       </c>
       <c r="C2">
         <v>3.7890000000000001</v>
@@ -522,13 +529,13 @@
         <v>1.5309999999999999</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>473.25</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>218.75</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>427.5</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -557,13 +564,16 @@
         <v>0.58499999999999996</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <f>1/12 *B3*(1.45^2 + 0.225^2)</f>
+        <v>136.561953125</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <f>1/12 *B3*(2.8^2 + 0.225^2)</f>
+        <v>500.46289062499994</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <f>1/12 *B3*(2.8^2 + 0.8^2)</f>
+        <v>537.84399999999994</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -577,7 +587,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4">
         <v>306</v>
@@ -612,7 +622,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>188.8</v>
@@ -647,19 +657,19 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B6">
         <v>24.1</v>
       </c>
       <c r="C6">
-        <v>3.8</v>
+        <v>3.3</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6">
-        <v>1.351</v>
+        <v>2.5129999999999999</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -682,19 +692,19 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="B7">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C7">
-        <v>2.5</v>
+        <v>3.4</v>
       </c>
       <c r="D7">
         <v>0</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>2.5129999999999999</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -717,19 +727,19 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B8">
-        <v>286.76799999999997</v>
+        <v>39.799999999999997</v>
       </c>
       <c r="C8">
-        <v>0.875</v>
+        <v>2.5</v>
       </c>
       <c r="D8">
         <v>0</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -752,19 +762,19 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="B9">
-        <v>16.309999999999999</v>
+        <v>12</v>
       </c>
       <c r="C9">
-        <v>2.0190000000000001</v>
+        <v>2.8</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -787,13 +797,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B10">
-        <v>16.399999999999999</v>
+        <v>286.76799999999997</v>
       </c>
       <c r="C10">
-        <v>0.56999999999999995</v>
+        <v>0.8</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -822,19 +832,19 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B11">
-        <v>53.87</v>
+        <v>16.309999999999999</v>
       </c>
       <c r="C11">
-        <v>3.1619999999999999</v>
+        <v>2.0190000000000001</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -857,19 +867,19 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12">
-        <v>5.25</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="C12">
-        <v>0.25</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -892,19 +902,19 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B13">
-        <v>50</v>
+        <v>53.87</v>
       </c>
       <c r="C13">
-        <v>5</v>
+        <v>3.1619999999999999</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13">
-        <v>2.5129999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -927,19 +937,19 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B14">
-        <v>20</v>
+        <v>5.25</v>
       </c>
       <c r="C14">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -962,19 +972,19 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B15">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="C15">
-        <v>1.75</v>
+        <v>5</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15">
-        <v>0.4</v>
+        <v>2.5129999999999999</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -997,19 +1007,19 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="B16">
-        <v>1.25</v>
+        <v>20</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -1032,19 +1042,19 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B17">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C17">
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="F17">
         <v>0</v>
@@ -1067,19 +1077,19 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B18">
-        <v>50</v>
+        <v>1.25</v>
       </c>
       <c r="C18">
-        <v>2.02</v>
+        <v>1</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18">
-        <v>2.1</v>
+        <v>1</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -1102,19 +1112,19 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B19">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="D19">
         <v>0</v>
       </c>
       <c r="E19">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="F19">
         <v>0</v>
@@ -1137,19 +1147,19 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B20">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="C20">
-        <v>4.4909999999999997</v>
+        <v>2.02</v>
       </c>
       <c r="D20">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="E20">
-        <v>1.020119</v>
+        <v>2.1</v>
       </c>
       <c r="F20">
         <v>0</v>
@@ -1172,19 +1182,19 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B21">
-        <v>104.65</v>
+        <v>72</v>
       </c>
       <c r="C21">
-        <v>4.476</v>
+        <v>3</v>
       </c>
       <c r="D21">
-        <v>-0.33500000000000002</v>
+        <v>0</v>
       </c>
       <c r="E21">
-        <v>0.97011899999999995</v>
+        <v>0.1</v>
       </c>
       <c r="F21">
         <v>0</v>
@@ -1207,19 +1217,19 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B22">
-        <v>104.65</v>
+        <v>120</v>
       </c>
       <c r="C22">
-        <v>3.8959999999999999</v>
+        <v>4.4909999999999997</v>
       </c>
       <c r="D22">
-        <v>-0.33500000000000002</v>
+        <v>0.3</v>
       </c>
       <c r="E22">
-        <v>0.97011899999999995</v>
+        <v>1.020119</v>
       </c>
       <c r="F22">
         <v>0</v>
@@ -1242,19 +1252,19 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B23">
-        <v>128.1</v>
+        <v>104.65</v>
       </c>
       <c r="C23">
-        <v>5.0410000000000004</v>
+        <v>4.476</v>
       </c>
       <c r="D23">
-        <v>-0.35</v>
+        <v>-0.33500000000000002</v>
       </c>
       <c r="E23">
-        <v>1.320119</v>
+        <v>0.97011899999999995</v>
       </c>
       <c r="F23">
         <v>0</v>
@@ -1277,19 +1287,19 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B24">
-        <v>45</v>
+        <v>104.65</v>
       </c>
       <c r="C24">
-        <v>4.4000000000000004</v>
+        <v>3.8959999999999999</v>
       </c>
       <c r="D24">
-        <v>0.6</v>
+        <v>-0.33500000000000002</v>
       </c>
       <c r="E24">
-        <v>1.35</v>
+        <v>0.97011899999999995</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1312,19 +1322,19 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B25">
-        <v>15</v>
+        <v>128.1</v>
       </c>
       <c r="C25">
-        <v>4.2</v>
+        <v>5.0410000000000004</v>
       </c>
       <c r="D25">
-        <v>0</v>
+        <v>-0.35</v>
       </c>
       <c r="E25">
-        <v>1.35</v>
+        <v>1.320119</v>
       </c>
       <c r="F25">
         <v>0</v>
@@ -1347,16 +1357,16 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B26">
-        <v>128.1</v>
+        <v>45</v>
       </c>
       <c r="C26">
-        <v>1.75</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="D26">
-        <v>-0.35</v>
+        <v>0.6</v>
       </c>
       <c r="E26">
         <v>1.35</v>
@@ -1382,36 +1392,106 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B27">
+        <v>15</v>
+      </c>
+      <c r="C27">
+        <v>4.2</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>1.35</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>0</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28">
+        <v>128.1</v>
+      </c>
+      <c r="C28">
+        <v>1.75</v>
+      </c>
+      <c r="D28">
+        <v>-0.35</v>
+      </c>
+      <c r="E28">
+        <v>1.35</v>
+      </c>
+      <c r="F28">
+        <v>0</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29">
         <v>104.65</v>
       </c>
-      <c r="C27">
+      <c r="C29">
         <v>1.75</v>
       </c>
-      <c r="D27">
+      <c r="D29">
         <v>0.33500000000000002</v>
       </c>
-      <c r="E27">
+      <c r="E29">
         <v>0.97011899999999995</v>
       </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-      <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="H27">
-        <v>0</v>
-      </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
-      <c r="J27">
-        <v>0</v>
-      </c>
-      <c r="K27">
+      <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
         <v>0</v>
       </c>
     </row>

</xml_diff>